<commit_message>
7. update silkscreen  and plane clearance
</commit_message>
<xml_diff>
--- a/Reference design documents/Design and component selection sheet.xlsx
+++ b/Reference design documents/Design and component selection sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\QRBOTS\PCB Projects\Nvidia_carrier_board_buck_converter\Reference design documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C253463E-7F06-42E3-89B5-5D0FE0CD609A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91D55952-2AA4-44CB-A4C7-9E8E3B452DF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="12240" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="150">
   <si>
     <t>LM61495-Q1</t>
   </si>
@@ -437,6 +437,57 @@
   </si>
   <si>
     <t>Calculator</t>
+  </si>
+  <si>
+    <t>Edge plating reference</t>
+  </si>
+  <si>
+    <t>Link</t>
+  </si>
+  <si>
+    <t>Top and bottom ground pour</t>
+  </si>
+  <si>
+    <t>pull out 20mils from board edge</t>
+  </si>
+  <si>
+    <t>Inner ground and power layers</t>
+  </si>
+  <si>
+    <t>MOSFET power dissipation calculation</t>
+  </si>
+  <si>
+    <t>Layer stack</t>
+  </si>
+  <si>
+    <t>Mosfet conduction loss</t>
+  </si>
+  <si>
+    <t>Rdson, max = 3.4m ohm</t>
+  </si>
+  <si>
+    <t>I max = 10A</t>
+  </si>
+  <si>
+    <t>Power loss = 0.34W</t>
+  </si>
+  <si>
+    <t>Temperature rise</t>
+  </si>
+  <si>
+    <t>Ambient temperature = 30 °C</t>
+  </si>
+  <si>
+    <t>Junction temperature  = 50.4 °C</t>
+  </si>
+  <si>
+    <t>IPC class 2 via plating thickness</t>
+  </si>
+  <si>
+    <t>0.02mm / 0.78mils</t>
+  </si>
+  <si>
+    <t>pull in 25 mils from board edge</t>
   </si>
 </sst>
 </file>
@@ -463,7 +514,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -500,6 +551,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -529,7 +586,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
@@ -546,6 +603,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -575,7 +634,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>312420</xdr:colOff>
+      <xdr:colOff>99060</xdr:colOff>
       <xdr:row>40</xdr:row>
       <xdr:rowOff>121920</xdr:rowOff>
     </xdr:to>
@@ -745,22 +804,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>45720</xdr:colOff>
-      <xdr:row>55</xdr:row>
-      <xdr:rowOff>7621</xdr:rowOff>
+      <xdr:colOff>106681</xdr:colOff>
+      <xdr:row>112</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>601980</xdr:colOff>
-      <xdr:row>75</xdr:row>
-      <xdr:rowOff>131023</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>147897</xdr:colOff>
+      <xdr:row>135</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Picture 5">
+        <xdr:cNvPr id="7" name="Picture 6">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{170371CE-50BE-53F6-1A76-680074F13452}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{81A9DA63-9BBC-E692-CA44-CD5B80285481}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -776,8 +835,228 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="45720" y="10066021"/>
-          <a:ext cx="11361420" cy="3781002"/>
+          <a:off x="106681" y="22898100"/>
+          <a:ext cx="2982536" cy="4168140"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>94</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>20321</xdr:colOff>
+      <xdr:row>96</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Picture 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F0517605-7346-8A40-042C-88D01DE2777F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2118361" y="17190720"/>
+          <a:ext cx="1849120" cy="426720"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>586740</xdr:colOff>
+      <xdr:row>93</xdr:row>
+      <xdr:rowOff>129540</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>68580</xdr:colOff>
+      <xdr:row>99</xdr:row>
+      <xdr:rowOff>132984</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Picture 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0C76D5AE-C847-1BD5-22E4-17FD6C513026}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5753100" y="17137380"/>
+          <a:ext cx="5730240" cy="1100724"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>167640</xdr:colOff>
+      <xdr:row>99</xdr:row>
+      <xdr:rowOff>121920</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>580389</xdr:colOff>
+      <xdr:row>101</xdr:row>
+      <xdr:rowOff>175260</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="Picture 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8DA1ECE5-6E4E-AA8B-7BB3-E028E75AAEAD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5943600" y="18227040"/>
+          <a:ext cx="1708149" cy="419100"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>411480</xdr:colOff>
+      <xdr:row>99</xdr:row>
+      <xdr:rowOff>137160</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>320303</xdr:colOff>
+      <xdr:row>102</xdr:row>
+      <xdr:rowOff>36</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="11" name="Picture 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2EBC2355-EEB2-D8A7-CC1C-1604B155D5DF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8092440" y="18242280"/>
+          <a:ext cx="3033023" cy="411516"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>76201</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>129540</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>266701</xdr:colOff>
+      <xdr:row>71</xdr:row>
+      <xdr:rowOff>105044</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="13" name="Picture 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{921B1AF9-CCAF-495C-DEC6-CC99E7B29480}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="76201" y="10005060"/>
+          <a:ext cx="9380220" cy="3084464"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1446,10 +1725,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DAB2649-7B4C-4B3E-90CE-6D62D92ECE20}">
-  <dimension ref="A1:U79"/>
+  <dimension ref="A1:U111"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.21875" customWidth="1"/>
+    <col min="1" max="1" width="19.33203125" customWidth="1"/>
     <col min="2" max="2" width="14.6640625" customWidth="1"/>
     <col min="9" max="9" width="5.88671875" customWidth="1"/>
     <col min="10" max="10" width="13" customWidth="1"/>
@@ -1787,7 +2066,9 @@
         <v>131</v>
       </c>
       <c r="B54" s="4"/>
-      <c r="C54" s="4"/>
+      <c r="C54" s="13" t="s">
+        <v>132</v>
+      </c>
       <c r="D54" s="4"/>
       <c r="E54" s="4"/>
       <c r="F54" s="4"/>
@@ -1807,20 +2088,159 @@
       <c r="T54" s="4"/>
       <c r="U54" s="4"/>
     </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A79" s="2" t="s">
-        <v>132</v>
-      </c>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A74" t="s">
+        <v>147</v>
+      </c>
+      <c r="C74" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="82" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A82" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="B82" s="4"/>
+      <c r="C82" s="4"/>
+      <c r="D82" s="4"/>
+      <c r="E82" s="4"/>
+      <c r="F82" s="4"/>
+      <c r="G82" s="4"/>
+      <c r="H82" s="4"/>
+      <c r="I82" s="4"/>
+      <c r="J82" s="4"/>
+      <c r="K82" s="4"/>
+      <c r="L82" s="4"/>
+      <c r="M82" s="4"/>
+      <c r="N82" s="4"/>
+      <c r="O82" s="4"/>
+      <c r="P82" s="4"/>
+      <c r="Q82" s="4"/>
+      <c r="R82" s="4"/>
+      <c r="S82" s="4"/>
+      <c r="T82" s="4"/>
+      <c r="U82" s="4"/>
+    </row>
+    <row r="84" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A84" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="87" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A87" t="s">
+        <v>135</v>
+      </c>
+      <c r="C87" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="89" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A89" t="s">
+        <v>137</v>
+      </c>
+      <c r="C89" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="93" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A93" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="B93" s="4"/>
+      <c r="C93" s="4"/>
+      <c r="D93" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="E93" s="4"/>
+      <c r="F93" s="4"/>
+      <c r="G93" s="4"/>
+      <c r="H93" s="4"/>
+      <c r="I93" s="4"/>
+      <c r="J93" s="4"/>
+      <c r="K93" s="4"/>
+      <c r="L93" s="4"/>
+      <c r="M93" s="4"/>
+      <c r="N93" s="4"/>
+      <c r="O93" s="4"/>
+      <c r="P93" s="4"/>
+      <c r="Q93" s="4"/>
+      <c r="R93" s="4"/>
+      <c r="S93" s="4"/>
+      <c r="T93" s="4"/>
+      <c r="U93" s="4"/>
+    </row>
+    <row r="95" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A95" s="12" t="s">
+        <v>140</v>
+      </c>
+      <c r="B95" s="12"/>
+      <c r="G95" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="H95" s="12"/>
+    </row>
+    <row r="98" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A98" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="99" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A99" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="100" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A100" s="10" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="105" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="H105" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="107" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="H107" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="I107" s="10"/>
+      <c r="J107" s="10"/>
+    </row>
+    <row r="111" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A111" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="B111" s="4"/>
+      <c r="C111" s="4"/>
+      <c r="D111" s="4"/>
+      <c r="E111" s="4"/>
+      <c r="F111" s="4"/>
+      <c r="G111" s="4"/>
+      <c r="H111" s="4"/>
+      <c r="I111" s="4"/>
+      <c r="J111" s="4"/>
+      <c r="K111" s="4"/>
+      <c r="L111" s="4"/>
+      <c r="M111" s="4"/>
+      <c r="N111" s="4"/>
+      <c r="O111" s="4"/>
+      <c r="P111" s="4"/>
+      <c r="Q111" s="4"/>
+      <c r="R111" s="4"/>
+      <c r="S111" s="4"/>
+      <c r="T111" s="4"/>
+      <c r="U111" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A4:B4"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A79" r:id="rId1" xr:uid="{46F32321-A5C6-421E-AB70-91FC5CE86D01}"/>
+    <hyperlink ref="C54" r:id="rId1" xr:uid="{46F32321-A5C6-421E-AB70-91FC5CE86D01}"/>
+    <hyperlink ref="A84" r:id="rId2" xr:uid="{298E5665-16AF-481C-869E-508CC97A6171}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId2"/>
+  <drawing r:id="rId3"/>
 </worksheet>
 </file>
 

</xml_diff>